<commit_message>
Added COs Lab and Classroom information in Excel file
</commit_message>
<xml_diff>
--- a/C6/Lab Photos with names/Lab information.xlsx
+++ b/C6/Lab Photos with names/Lab information.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21840" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Classroom info" sheetId="1" r:id="rId1"/>
+    <sheet name="Labs Info CO" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,9 +19,175 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
+  <si>
+    <t>Sr. No</t>
+  </si>
+  <si>
+    <t>Classroom No.</t>
+  </si>
+  <si>
+    <t>Board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duel Bench, Seating Capacity </t>
+  </si>
+  <si>
+    <t>Tube-light,Fan</t>
+  </si>
+  <si>
+    <t>Area Sq. m</t>
+  </si>
+  <si>
+    <t>Remark</t>
+  </si>
+  <si>
+    <t>Class Room - 108</t>
+  </si>
+  <si>
+    <t>First Year Class Room ( Main Building )</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Duel Bench (60+ nos.)</t>
+  </si>
+  <si>
+    <t>As Per AICTE Norms</t>
+  </si>
+  <si>
+    <t>Class Room - 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second Year Class Room (Computer Engg. Building ) </t>
+  </si>
+  <si>
+    <t>Class Room – 3 Third Year Class Room (Computer Engg. Building )</t>
+  </si>
+  <si>
+    <t>Class Room – 201</t>
+  </si>
+  <si>
+    <t>Drawing Hall ( Main Building )</t>
+  </si>
+  <si>
+    <t>Wooden Drawing desks with stools (70+ nos.)</t>
+  </si>
+  <si>
+    <t>Tutorial Room ( Main Building )</t>
+  </si>
+  <si>
+    <t>Duel Bench (15+ nos.)</t>
+  </si>
+  <si>
+    <t>Name of Laboratory</t>
+  </si>
+  <si>
+    <t>Name of Important Equipment/Facility</t>
+  </si>
+  <si>
+    <t>No. of Students Per Batch</t>
+  </si>
+  <si>
+    <t>Basic Programming Laboratory</t>
+  </si>
+  <si>
+    <t>21 Desktop PCs with Cushioned Chairs and CCTV cameras</t>
+  </si>
+  <si>
+    <t>20 Students</t>
+  </si>
+  <si>
+    <t>1- Smart Board, 1- T,V Set, 1- AC, Epson MFP Printer</t>
+  </si>
+  <si>
+    <t>Android App Development Laboratory</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Students</t>
+    </r>
+  </si>
+  <si>
+    <t>1- Smart Board, 1- AC, ALTOS Server</t>
+  </si>
+  <si>
+    <t>Software Engineering Laboratory</t>
+  </si>
+  <si>
+    <t>24 Desktop PCs with Cushioned Chairs and CCTV cameras</t>
+  </si>
+  <si>
+    <t>1- AC Facility, 1- Wheel Chair</t>
+  </si>
+  <si>
+    <t>Web Development Laboratory</t>
+  </si>
+  <si>
+    <t>1- AC, 1- Wheel Chair</t>
+  </si>
+  <si>
+    <t>Advanced Programming Laboratory</t>
+  </si>
+  <si>
+    <t>30 Desktop PCs with Cushioned Chairs and CCTV cameras</t>
+  </si>
+  <si>
+    <t>Unix/OS Laboratory</t>
+  </si>
+  <si>
+    <t>1- AC,1-Cup-board,1-White board</t>
+  </si>
+  <si>
+    <t>Hardware and Networking Laboratory</t>
+  </si>
+  <si>
+    <t>Desktop PCs with Chairs and Hardware Kits</t>
+  </si>
+  <si>
+    <t>Physics Laboratory</t>
+  </si>
+  <si>
+    <t>Joules calorimeter, Searle’s apparatus, Photocell, Vernier calliper, Micro meter screw gauge</t>
+  </si>
+  <si>
+    <t>Shared Usage</t>
+  </si>
+  <si>
+    <t>Chemistry Laboratory</t>
+  </si>
+  <si>
+    <t>Electric oven, Muffle furnace, PH meter.</t>
+  </si>
+  <si>
+    <t>Language Laboratory</t>
+  </si>
+  <si>
+    <t>24 Desktop PCs with Headset</t>
+  </si>
+  <si>
+    <t>Digital Electronics Laboratory</t>
+  </si>
+  <si>
+    <t>Basic Electrical Engineering Laboratory</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +195,53 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEECE1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -45,12 +249,135 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -323,7 +650,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -331,9 +658,429 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" customWidth="1"/>
+    <col min="3" max="7" width="14.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="G2" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="10"/>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="10"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="11"/>
+      <c r="G4" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10"/>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="10"/>
+    </row>
+    <row r="6" spans="1:7" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>4</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="10"/>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" spans="1:7" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" customWidth="1"/>
+    <col min="3" max="3" width="55.85546875" customWidth="1"/>
+    <col min="4" max="5" width="35.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14">
+        <v>2</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="14">
+        <v>5</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>6</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
+        <v>7</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="14"/>
+    </row>
+    <row r="9" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="14">
+        <v>8</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="14">
+        <v>9</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>10</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>12</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="50" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>